<commit_message>
problems on palindrome number
</commit_message>
<xml_diff>
--- a/Python code statements.xlsx
+++ b/Python code statements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\Python Programming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10EC6AB2-75E2-4D0B-8615-C6BD866E1929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3291FB92-A049-4E04-A118-1EAD4E1F1B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{004C20B9-D5AA-4773-B689-5502DB922027}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{004C20B9-D5AA-4773-B689-5502DB922027}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>print Jay Ganesh</t>
   </si>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>Printing digits in a number</t>
+  </si>
+  <si>
+    <t>Even Odd digit sum and difference</t>
+  </si>
+  <si>
+    <t>Palindrome number</t>
   </si>
 </sst>
 </file>
@@ -412,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C0B0B21-D0B4-41AD-AEDB-F9C0466522F6}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.28515625" bestFit="1" customWidth="1"/>
@@ -463,6 +469,16 @@
         <v>8</v>
       </c>
     </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>